<commit_message>
fix: ajustes nos nomes e testes nos usuarios
</commit_message>
<xml_diff>
--- a/Dados do Responsável do Setor.xlsx
+++ b/Dados do Responsável do Setor.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <x:si>
     <x:t xml:space="preserve">ID</x:t>
   </x:si>
@@ -139,6 +139,18 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">administrativo</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">dasdasd</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">qwe.qwe</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">asd@ggmail.com</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">sistemas</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -235,8 +247,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q3" insertRow="1" totalsRowShown="0">
-  <x:autoFilter ref="A1:Q3"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q4" insertRow="1" totalsRowShown="0">
+  <x:autoFilter ref="A1:Q4"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" uniqueName="1" name="ID" dataDxfId="0"/>
     <x:tableColumn id="2" uniqueName="2" name="Hora de início" dataDxfId="3"/>
@@ -730,11 +742,60 @@
         <x:v>37</x:v>
       </x:c>
     </x:row>
+    <x:row r="4" hidden="0">
+      <x:c r="A4">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B4" s="2">
+        <x:v>46097.6920486111</x:v>
+      </x:c>
+      <x:c r="C4" s="2">
+        <x:v>46097.6928935185</x:v>
+      </x:c>
+      <x:c r="D4" s="10" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E4" s="10" t="s"/>
+      <x:c r="F4" s="2"/>
+      <x:c r="G4" s="10" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="H4" s="7" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="I4" s="10" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J4" s="10" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="K4" s="10" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L4" s="7" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="M4" s="10" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="N4" s="7" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="O4" s="10" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="P4" s="10" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="Q4" s="10" t="s">
+        <x:v>41</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <x:tableParts count="1">
-    <x:tablePart r:id="R85a465e9fb534f2b"/>
+    <x:tablePart r:id="Rd2dbf3d00cb94be3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
reajuste na ordem dos campos
</commit_message>
<xml_diff>
--- a/Dados do Responsável do Setor.xlsx
+++ b/Dados do Responsável do Setor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qinzen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{95448ABA-98DB-46AA-857C-5EF6458B4E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2677DE22-B0B1-4E7B-9AE3-67D22EE277A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="236">
   <si>
     <t>Id</t>
   </si>
@@ -257,6 +257,83 @@
     <t>Há mais servidores para cadastrar?9</t>
   </si>
   <si>
+    <t>Nome do servidor10</t>
+  </si>
+  <si>
+    <t>Matrícula do servidor10</t>
+  </si>
+  <si>
+    <t>Login de rede10</t>
+  </si>
+  <si>
+    <t>E-mail institucional10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coordenação do servidor
+</t>
+  </si>
+  <si>
+    <t>Nome do servidor11</t>
+  </si>
+  <si>
+    <t>Matrícula do servidor11</t>
+  </si>
+  <si>
+    <t>Login de rede11</t>
+  </si>
+  <si>
+    <t>E-mail institucional11</t>
+  </si>
+  <si>
+    <t>Coordenação do servidor10</t>
+  </si>
+  <si>
+    <t>Nome do servidor12</t>
+  </si>
+  <si>
+    <t>Matrícula do servidor12</t>
+  </si>
+  <si>
+    <t>Login de rede12</t>
+  </si>
+  <si>
+    <t>E-mail institucional14</t>
+  </si>
+  <si>
+    <t>Coordenação do servidor12</t>
+  </si>
+  <si>
+    <t>Nome do servidor13</t>
+  </si>
+  <si>
+    <t>Matrícula do servidor13</t>
+  </si>
+  <si>
+    <t>Login de rede13</t>
+  </si>
+  <si>
+    <t>E-mail institucional12</t>
+  </si>
+  <si>
+    <t>Coordenação do servidor
+1</t>
+  </si>
+  <si>
+    <t>Nome do servidor14</t>
+  </si>
+  <si>
+    <t>Matrícula do servidor14</t>
+  </si>
+  <si>
+    <t>Login de rede14</t>
+  </si>
+  <si>
+    <t>E-mail institucional13</t>
+  </si>
+  <si>
+    <t>Coordenação do servidor11</t>
+  </si>
+  <si>
     <t>anonymous</t>
   </si>
   <si>
@@ -633,6 +710,42 @@
   </si>
   <si>
     <t>dfgdfgdfgd</t>
+  </si>
+  <si>
+    <t>resrte</t>
+  </si>
+  <si>
+    <t>asdas</t>
+  </si>
+  <si>
+    <t>testado@gmail.com</t>
+  </si>
+  <si>
+    <t>depart-teste</t>
+  </si>
+  <si>
+    <t>teste-subsecretaria</t>
+  </si>
+  <si>
+    <t>testtt</t>
+  </si>
+  <si>
+    <t>tes.tt</t>
+  </si>
+  <si>
+    <t>teste@asdasd</t>
+  </si>
+  <si>
+    <t>jkljç</t>
+  </si>
+  <si>
+    <t>çjkçjkç</t>
+  </si>
+  <si>
+    <t>jkljkljkl</t>
+  </si>
+  <si>
+    <t>ljkljkl</t>
   </si>
 </sst>
 </file>
@@ -668,19 +781,97 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="71">
+  <dxfs count="96">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -908,10 +1099,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:BU12" totalsRowShown="0">
-  <autoFilter ref="A1:BU12" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="73">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="70">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="OfficeForms.Table" displayName="OfficeForms.Table" ref="A1:CT13" totalsRowShown="0">
+  <autoFilter ref="A1:CT13" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="98">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id" dataDxfId="95">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="id"/>
@@ -932,493 +1123,668 @@
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="69">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="94">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="responder"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Nome" dataDxfId="68">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Nome" dataDxfId="93">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="responderName"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Nome do responsável" dataDxfId="67">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Nome do responsável" dataDxfId="92">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r6aad2d12215f4c2b81136d9277535010"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Matrícula do responsável" dataDxfId="66">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Matrícula do responsável" dataDxfId="91">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r9973d738f9724a3a8e2cbd5d103c0be7"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Login de rede do responsável" dataDxfId="65">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Login de rede do responsável" dataDxfId="90">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r82497e02c592432689fff1cddbb6c911"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="E-mail institucional do responsável" dataDxfId="64">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="E-mail institucional do responsável" dataDxfId="89">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r6fb60a8ac9744c1787bf1c8870f93fef"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Departamento" dataDxfId="63">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Departamento" dataDxfId="88">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r1d1c6f03c2824b5d93f2133b641310a1"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="72" xr3:uid="{FEA36EAB-8BA3-45A3-9C4B-0652E253593D}" name="Este departamento está subordinado à alguma Subsecretaria?" dataDxfId="62">
+    <tableColumn id="72" xr3:uid="{FEA36EAB-8BA3-45A3-9C4B-0652E253593D}" name="Este departamento está subordinado à alguma Subsecretaria?" dataDxfId="87">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r2498731ab00f4da28f82ffdb063b6d21"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="73" xr3:uid="{929C21BA-8618-4A13-933D-93CDCF31E314}" name="Informe o nome da Subsecretaria" dataDxfId="61">
+    <tableColumn id="73" xr3:uid="{929C21BA-8618-4A13-933D-93CDCF31E314}" name="Informe o nome da Subsecretaria" dataDxfId="86">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r1a9c813d9b0a445d9ce4a40e335039c3"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Quantidade de servidores" dataDxfId="60">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Quantidade de servidores" dataDxfId="85">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r604ffbe803bc446b81030ca302b10887"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Nome do servidor" dataDxfId="59">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Nome do servidor" dataDxfId="84">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r3e8592c939d84b68a61cf5c3f39622a9"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Matrícula do servidor" dataDxfId="58">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Matrícula do servidor" dataDxfId="83">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rcfbd5a4544584b5ea489f0e9ae246228"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Login de rede" dataDxfId="57">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Login de rede" dataDxfId="82">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r3c71372d9009413fbf441e6dc6f828d7"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="E-mail institucional" dataDxfId="56">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="E-mail institucional" dataDxfId="81">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r9e917fad469f49f29ac2e1197b37e402"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Coordenação do servidor" dataDxfId="55">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Coordenação do servidor" dataDxfId="80">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r93c1649fb86c4e9ab340e69c3ba1a1a5"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{19D456CB-7091-432A-8467-820AE92013AA}" name="Há mais servidores para cadastrar?" dataDxfId="54">
+    <tableColumn id="17" xr3:uid="{19D456CB-7091-432A-8467-820AE92013AA}" name="Há mais servidores para cadastrar?" dataDxfId="79">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rd3718218eabe4f9f8b1823158151b48b"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{03178331-B7E3-4C8A-84F7-587CACABB3E2}" name="Nome do servidor1" dataDxfId="53">
+    <tableColumn id="18" xr3:uid="{03178331-B7E3-4C8A-84F7-587CACABB3E2}" name="Nome do servidor1" dataDxfId="78">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r0597e6fe86bc4cffb6167876bd0cd253"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{5CFDF991-3E82-4E53-AFAD-E72B9382D6CE}" name="Matrícula do servidor1" dataDxfId="52">
+    <tableColumn id="19" xr3:uid="{5CFDF991-3E82-4E53-AFAD-E72B9382D6CE}" name="Matrícula do servidor1" dataDxfId="77">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r53b03e51c8bf49b5a5e4b42d18affd6f"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{6A9EFF49-4DD0-41EA-82A9-4773A39B44FD}" name="Login de rede1" dataDxfId="51">
+    <tableColumn id="20" xr3:uid="{6A9EFF49-4DD0-41EA-82A9-4773A39B44FD}" name="Login de rede1" dataDxfId="76">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r983fc2db42244b5396c1f6be5b7409fd"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{D7CF2C48-2417-4BB1-B082-F60A8C2F8BB6}" name="E-mail institucional1" dataDxfId="50">
+    <tableColumn id="21" xr3:uid="{D7CF2C48-2417-4BB1-B082-F60A8C2F8BB6}" name="E-mail institucional1" dataDxfId="75">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="ree488357bd4e4964b5b4e546a163d02f"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{B2F68F06-E772-4BD5-96C6-4BC7ABFB4BC1}" name="Coordenação do servidor1" dataDxfId="49">
+    <tableColumn id="22" xr3:uid="{B2F68F06-E772-4BD5-96C6-4BC7ABFB4BC1}" name="Coordenação do servidor1" dataDxfId="74">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r06868787963d4797926d351f1f18621a"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{C5F698B6-607C-4076-B856-0350E486B9FF}" name="Há mais servidores para cadastrar?1" dataDxfId="48">
+    <tableColumn id="23" xr3:uid="{C5F698B6-607C-4076-B856-0350E486B9FF}" name="Há mais servidores para cadastrar?1" dataDxfId="73">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r82d196bfe54d4104b6aa2b497b059817"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{B6304EA7-53CC-49F5-B8A5-0088EF5307BB}" name="Nome do servidor2" dataDxfId="47">
+    <tableColumn id="24" xr3:uid="{B6304EA7-53CC-49F5-B8A5-0088EF5307BB}" name="Nome do servidor2" dataDxfId="72">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rba5b7bd63d2f48f4be5efdc095bf1b51"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="25" xr3:uid="{3E779B42-014F-476C-809B-8BAF0174B147}" name="Matrícula do servidor2" dataDxfId="46">
+    <tableColumn id="25" xr3:uid="{3E779B42-014F-476C-809B-8BAF0174B147}" name="Matrícula do servidor2" dataDxfId="71">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r2e314bd5332a46298b0ebd2543ed582e"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="26" xr3:uid="{4D2DB918-8F71-4F3E-B268-79300B4BAD5A}" name="Login de rede2" dataDxfId="45">
+    <tableColumn id="26" xr3:uid="{4D2DB918-8F71-4F3E-B268-79300B4BAD5A}" name="Login de rede2" dataDxfId="70">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r2686778ea9cc4c84bbb8cdefffd8f603"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="27" xr3:uid="{DB373380-088F-4EB8-9BA3-E0D285BB876C}" name="E-mail institucional2" dataDxfId="44">
+    <tableColumn id="27" xr3:uid="{DB373380-088F-4EB8-9BA3-E0D285BB876C}" name="E-mail institucional2" dataDxfId="69">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rbfc6e99494d14c479ae13e3405ae89b5"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{82E8C4FF-835C-4A32-9AB0-96EDE1652D71}" name="Coordenação do servidor2" dataDxfId="43">
+    <tableColumn id="28" xr3:uid="{82E8C4FF-835C-4A32-9AB0-96EDE1652D71}" name="Coordenação do servidor2" dataDxfId="68">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r884b25d531844f5a9469c788b7da53b2"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{18084BCB-5944-41C8-912A-76761AB58B9C}" name="Há mais servidores para cadastrar?2" dataDxfId="42">
+    <tableColumn id="29" xr3:uid="{18084BCB-5944-41C8-912A-76761AB58B9C}" name="Há mais servidores para cadastrar?2" dataDxfId="67">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="re079310821074189a670023a877d1939"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="30" xr3:uid="{8BC63F8E-6844-473D-A974-DC5DED1B62CC}" name="Nome do servidor3" dataDxfId="41">
+    <tableColumn id="30" xr3:uid="{8BC63F8E-6844-473D-A974-DC5DED1B62CC}" name="Nome do servidor3" dataDxfId="66">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rf0caf971ebc1405598ecae18f62c7691"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="31" xr3:uid="{6B760FF7-F590-40B2-8848-551F353DF084}" name="Matrícula do servidor3" dataDxfId="40">
+    <tableColumn id="31" xr3:uid="{6B760FF7-F590-40B2-8848-551F353DF084}" name="Matrícula do servidor3" dataDxfId="65">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r11967a726b3b4c55a507a8372f3fa7f1"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="32" xr3:uid="{08C67F45-AB9B-483F-B59E-CF5BD0912FF3}" name="Login de rede3" dataDxfId="39">
+    <tableColumn id="32" xr3:uid="{08C67F45-AB9B-483F-B59E-CF5BD0912FF3}" name="Login de rede3" dataDxfId="64">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r1125d616a4f548d4bb994f0157342638"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="33" xr3:uid="{39F24A1E-4259-48D5-940B-B43DCAE4A1BE}" name="E-mail institucional3" dataDxfId="38">
+    <tableColumn id="33" xr3:uid="{39F24A1E-4259-48D5-940B-B43DCAE4A1BE}" name="E-mail institucional3" dataDxfId="63">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="re3fb5f7090844f13bc7d007bef3ea0fa"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{781FD850-93F4-4B54-A362-48F9FF5D366D}" name="Coordenação do servidor3" dataDxfId="37">
+    <tableColumn id="34" xr3:uid="{781FD850-93F4-4B54-A362-48F9FF5D366D}" name="Coordenação do servidor3" dataDxfId="62">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rc161561ce20d4984bd4204dcbd9b4045"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="35" xr3:uid="{09866D5B-DF76-45FC-A586-607B35A05730}" name="Há mais servidores para cadastrar?3" dataDxfId="36">
+    <tableColumn id="35" xr3:uid="{09866D5B-DF76-45FC-A586-607B35A05730}" name="Há mais servidores para cadastrar?3" dataDxfId="61">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="re69a2538c16249d296c0a1f44722b065"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="36" xr3:uid="{E09668C6-E10A-445C-901B-50B863556332}" name="Nome do servidor4" dataDxfId="35">
+    <tableColumn id="36" xr3:uid="{E09668C6-E10A-445C-901B-50B863556332}" name="Nome do servidor4" dataDxfId="60">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rbbb16eea61804c828ebed41b43f6076b"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="37" xr3:uid="{03204F88-B744-4233-AB87-34908BDB7483}" name="Matrícula do servidor4" dataDxfId="34">
+    <tableColumn id="37" xr3:uid="{03204F88-B744-4233-AB87-34908BDB7483}" name="Matrícula do servidor4" dataDxfId="59">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r44abafa91e6b46e484648f052c601f64"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="38" xr3:uid="{4DF685B2-412C-4AB3-A459-66E372B6D871}" name="Login de rede4" dataDxfId="33">
+    <tableColumn id="38" xr3:uid="{4DF685B2-412C-4AB3-A459-66E372B6D871}" name="Login de rede4" dataDxfId="58">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rb2520f4fd3024c2883e6e3d5155105c8"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="39" xr3:uid="{56AB26EE-CAF2-4B79-A97C-DF36679FF2BE}" name="E-mail institucional4" dataDxfId="32">
+    <tableColumn id="39" xr3:uid="{56AB26EE-CAF2-4B79-A97C-DF36679FF2BE}" name="E-mail institucional4" dataDxfId="57">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="ra5cc7179312b462cb0c616afe9e7ad71"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="40" xr3:uid="{6A8F18CA-2B61-42BC-9955-8A81DFDAF5AD}" name="Coordenação do servidor4" dataDxfId="31">
+    <tableColumn id="40" xr3:uid="{6A8F18CA-2B61-42BC-9955-8A81DFDAF5AD}" name="Coordenação do servidor4" dataDxfId="56">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r399c904b38f5402ebd488d5638f666dc"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="41" xr3:uid="{B81321DF-5E5C-4257-9A2F-90705510D866}" name="Há mais servidores para cadastrar?4" dataDxfId="30">
+    <tableColumn id="41" xr3:uid="{B81321DF-5E5C-4257-9A2F-90705510D866}" name="Há mais servidores para cadastrar?4" dataDxfId="55">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r5e14e6148756474c9c4e1ba02fbc0845"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="42" xr3:uid="{FFED686C-2CAD-4282-ACE2-CFA49360A7FA}" name="Nome do servidor5" dataDxfId="29">
+    <tableColumn id="42" xr3:uid="{FFED686C-2CAD-4282-ACE2-CFA49360A7FA}" name="Nome do servidor5" dataDxfId="54">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r1b883b8e1c6240069c93e7323053017c"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="43" xr3:uid="{4A672424-95C1-408F-98AB-58FCB4321706}" name="Matrícula do servidor5" dataDxfId="28">
+    <tableColumn id="43" xr3:uid="{4A672424-95C1-408F-98AB-58FCB4321706}" name="Matrícula do servidor5" dataDxfId="53">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r45aa331aa8094877852a069ffa2cee22"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="44" xr3:uid="{B27BC188-2E17-4CF6-960F-EEC0AD9F064E}" name="Login de rede5" dataDxfId="27">
+    <tableColumn id="44" xr3:uid="{B27BC188-2E17-4CF6-960F-EEC0AD9F064E}" name="Login de rede5" dataDxfId="52">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="ra0ab63d795b342bab86b098b28be3a6f"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="45" xr3:uid="{851431DD-96BD-44CF-AFE1-E1DA0CE4C02D}" name="E-mail institucional5" dataDxfId="26">
+    <tableColumn id="45" xr3:uid="{851431DD-96BD-44CF-AFE1-E1DA0CE4C02D}" name="E-mail institucional5" dataDxfId="51">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r8590b92908744ef0afd13fb5bde1b17e"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="46" xr3:uid="{1BFAE9E3-9679-4BA5-B2F1-632FF2315E78}" name="Coordenação do servidor5" dataDxfId="25">
+    <tableColumn id="46" xr3:uid="{1BFAE9E3-9679-4BA5-B2F1-632FF2315E78}" name="Coordenação do servidor5" dataDxfId="50">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rf7e0ec5809c74d2c9771e57f7f5f3e80"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="47" xr3:uid="{7F0EDB25-1AF6-4C0D-87A8-BA6C4DF9D246}" name="Há mais servidores para cadastrar?5" dataDxfId="24">
+    <tableColumn id="47" xr3:uid="{7F0EDB25-1AF6-4C0D-87A8-BA6C4DF9D246}" name="Há mais servidores para cadastrar?5" dataDxfId="49">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r3dc708e38ab44ba6a5f2621278fa37ab"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="48" xr3:uid="{418E4BD4-9212-41EE-BDCB-1F6F2FF39E89}" name="Nome do servidor6" dataDxfId="23">
+    <tableColumn id="48" xr3:uid="{418E4BD4-9212-41EE-BDCB-1F6F2FF39E89}" name="Nome do servidor6" dataDxfId="48">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r30f16c8b6f864f47b0ca1d78b9015ff6"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="49" xr3:uid="{8F2396FA-8C74-40F5-801E-47DAC6710E44}" name="Matrícula do servidor6" dataDxfId="22">
+    <tableColumn id="49" xr3:uid="{8F2396FA-8C74-40F5-801E-47DAC6710E44}" name="Matrícula do servidor6" dataDxfId="47">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r5a2e020b04e94bed9d5190609ecc6af0"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="50" xr3:uid="{5E812DB0-4EF8-447B-ABFF-F0A78BEC1ACC}" name="Login de rede6" dataDxfId="21">
+    <tableColumn id="50" xr3:uid="{5E812DB0-4EF8-447B-ABFF-F0A78BEC1ACC}" name="Login de rede6" dataDxfId="46">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r142ee31b588349d7858d03993175e64a"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="51" xr3:uid="{0D401D20-838B-42AC-A6EE-92A6684F6F7E}" name="E-mail institucional6" dataDxfId="20">
+    <tableColumn id="51" xr3:uid="{0D401D20-838B-42AC-A6EE-92A6684F6F7E}" name="E-mail institucional6" dataDxfId="45">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r144a7a0b4485429b936852f57fe46545"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="52" xr3:uid="{11E07B0A-5ED6-435F-A34A-16E87318516F}" name="Coordenação do servidor6" dataDxfId="19">
+    <tableColumn id="52" xr3:uid="{11E07B0A-5ED6-435F-A34A-16E87318516F}" name="Coordenação do servidor6" dataDxfId="44">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r53d6f5cedcc944fd99ada40abf7279aa"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="53" xr3:uid="{CD6FAB8B-0D84-4EFE-B9E7-24BD2AAFC27F}" name="Há mais servidores para cadastrar?6" dataDxfId="18">
+    <tableColumn id="53" xr3:uid="{CD6FAB8B-0D84-4EFE-B9E7-24BD2AAFC27F}" name="Há mais servidores para cadastrar?6" dataDxfId="43">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r2aa04f51bd124ec0a5059bae66cc10e2"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="54" xr3:uid="{D9DF2645-9FFA-4624-8F36-44AA40936709}" name="Nome do servidor7" dataDxfId="17">
+    <tableColumn id="54" xr3:uid="{D9DF2645-9FFA-4624-8F36-44AA40936709}" name="Nome do servidor7" dataDxfId="42">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r7bc4dd35a5f64bd9962dbe75e5590280"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="55" xr3:uid="{FC99B652-454F-43AE-9432-0839CD2ABD4F}" name="Matrícula do servidor7" dataDxfId="16">
+    <tableColumn id="55" xr3:uid="{FC99B652-454F-43AE-9432-0839CD2ABD4F}" name="Matrícula do servidor7" dataDxfId="41">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r7101ec92084d4145917beb05269fc695"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="56" xr3:uid="{322331CF-9E99-4A00-8588-F902FEE63327}" name="Login de rede7" dataDxfId="15">
+    <tableColumn id="56" xr3:uid="{322331CF-9E99-4A00-8588-F902FEE63327}" name="Login de rede7" dataDxfId="40">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r98c454ffb7f64c0789eb73d04c88e0a7"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="57" xr3:uid="{6506AF0C-F916-46F3-8184-1F6B175EB896}" name="E-mail institucional7" dataDxfId="14">
+    <tableColumn id="57" xr3:uid="{6506AF0C-F916-46F3-8184-1F6B175EB896}" name="E-mail institucional7" dataDxfId="39">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r0ca7f3d37df1452fa6825f41138f6362"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="58" xr3:uid="{A91986F1-9C1E-4CEA-B35B-4F9B2DD79D4D}" name="Coordenação do servidor7" dataDxfId="13">
+    <tableColumn id="58" xr3:uid="{A91986F1-9C1E-4CEA-B35B-4F9B2DD79D4D}" name="Coordenação do servidor7" dataDxfId="38">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r4eeb0b946a6146bf9a5ef1b2a0566025"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="59" xr3:uid="{6ADBA388-5D41-4793-8B53-E88D29792E47}" name="Há mais servidores para cadastrar?7" dataDxfId="12">
+    <tableColumn id="59" xr3:uid="{6ADBA388-5D41-4793-8B53-E88D29792E47}" name="Há mais servidores para cadastrar?7" dataDxfId="37">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rb7d63a2919fe40068a8c0f916da15321"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="60" xr3:uid="{C6B48333-D431-4322-B0B6-8EAF47AE180A}" name="Nome do servidor8" dataDxfId="11">
+    <tableColumn id="60" xr3:uid="{C6B48333-D431-4322-B0B6-8EAF47AE180A}" name="Nome do servidor8" dataDxfId="36">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r95b3fb625ae242f9bcdb3c7d1771be37"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="61" xr3:uid="{08C814CE-743B-441B-90D6-007B39FBC9BF}" name="Matrícula do servidor8" dataDxfId="10">
+    <tableColumn id="61" xr3:uid="{08C814CE-743B-441B-90D6-007B39FBC9BF}" name="Matrícula do servidor8" dataDxfId="35">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r9b56dac29a974c318c0735ffebab0b8b"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="62" xr3:uid="{446C02D8-EC4E-4365-B5B6-7C7F4C942F8E}" name="Login de rede8" dataDxfId="9">
+    <tableColumn id="62" xr3:uid="{446C02D8-EC4E-4365-B5B6-7C7F4C942F8E}" name="Login de rede8" dataDxfId="34">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="rbe020e3fb76448489a838c3b22199a35"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="63" xr3:uid="{C9E3B7EC-E1E3-435E-AEFD-A2D820AFD55F}" name="E-mail institucional8" dataDxfId="8">
+    <tableColumn id="63" xr3:uid="{C9E3B7EC-E1E3-435E-AEFD-A2D820AFD55F}" name="E-mail institucional8" dataDxfId="33">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r2d1518605d5b416b977534fb6c360a07"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="64" xr3:uid="{2EE68F37-BD05-4443-9846-61328297CAA9}" name="Coordenação do servidor8" dataDxfId="7">
+    <tableColumn id="64" xr3:uid="{2EE68F37-BD05-4443-9846-61328297CAA9}" name="Coordenação do servidor8" dataDxfId="32">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r7a49244cad6a409c825dd3d169c8edb7"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="65" xr3:uid="{CE146896-6D46-47C1-8976-9B9B23A0692A}" name="Há mais servidores para cadastrar?8" dataDxfId="6">
+    <tableColumn id="65" xr3:uid="{CE146896-6D46-47C1-8976-9B9B23A0692A}" name="Há mais servidores para cadastrar?8" dataDxfId="31">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r8561c48b8999444b8a127cfd4d51cf50"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="66" xr3:uid="{B6C08122-7467-49AA-A717-4D6E29A05A46}" name="Nome do servidor9" dataDxfId="5">
+    <tableColumn id="66" xr3:uid="{B6C08122-7467-49AA-A717-4D6E29A05A46}" name="Nome do servidor9" dataDxfId="30">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r2dcebf95995e438e892bf6609682eabd"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="67" xr3:uid="{91E90836-C7BD-4B30-910C-9CDA606FE702}" name="Matrícula do servidor9" dataDxfId="4">
+    <tableColumn id="67" xr3:uid="{91E90836-C7BD-4B30-910C-9CDA606FE702}" name="Matrícula do servidor9" dataDxfId="29">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="ra8e547b3f64f4d0e8a125982fe1ba9db"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="68" xr3:uid="{A7B4A2CD-2248-4E53-8566-396E2B9D605C}" name="Login de rede9" dataDxfId="3">
+    <tableColumn id="68" xr3:uid="{A7B4A2CD-2248-4E53-8566-396E2B9D605C}" name="Login de rede9" dataDxfId="28">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r00340a0be2044a83a51f9eea148bda58"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="69" xr3:uid="{5C5D6FEE-BA6E-450E-904E-021830FF1CF7}" name="E-mail institucional9" dataDxfId="2">
+    <tableColumn id="69" xr3:uid="{5C5D6FEE-BA6E-450E-904E-021830FF1CF7}" name="E-mail institucional9" dataDxfId="27">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r6eaa922a3d88473e95ea6d008054b57b"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="70" xr3:uid="{1C48CC18-00C8-4047-88B7-90178AAEF2D8}" name="Coordenação do servidor9" dataDxfId="1">
+    <tableColumn id="70" xr3:uid="{1C48CC18-00C8-4047-88B7-90178AAEF2D8}" name="Coordenação do servidor9" dataDxfId="26">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r35a389d83a504d5cafb78198aaef06c9"/>
         </ext>
       </extLst>
     </tableColumn>
-    <tableColumn id="71" xr3:uid="{2035E222-CD93-4BBE-8C3D-2F6D4368ECCA}" name="Há mais servidores para cadastrar?9" dataDxfId="0">
+    <tableColumn id="71" xr3:uid="{2035E222-CD93-4BBE-8C3D-2F6D4368ECCA}" name="Há mais servidores para cadastrar?9" dataDxfId="25">
       <extLst>
         <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
           <xlmsforms:question id="r993ffb00f9924bcbb8f493f7869380b6"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="74" xr3:uid="{2B72DDB7-40EF-447D-AD25-1A98B6F49B87}" name="Nome do servidor10" dataDxfId="24">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="rac27fd054e3345469c7b9996b6af173a"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="75" xr3:uid="{FB1066A1-C475-4A1A-A980-D5ACF00FE7C6}" name="Matrícula do servidor10" dataDxfId="23">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r4256c493215a4a2097426ca815f3afda"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="76" xr3:uid="{078E9E47-C627-464C-AB35-1633B116CC57}" name="Login de rede10" dataDxfId="22">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r1a9fbbe7b2244704bb8ecc69f4bffeb4"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="77" xr3:uid="{16C21704-5F37-4720-A38C-165CB94BB52A}" name="E-mail institucional10" dataDxfId="21">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r3bcc0c0e808a46169ae8a8ea01caf5d4"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="78" xr3:uid="{B4778B1E-AAE7-43B8-8725-693DB6935860}" name="Coordenação do servidor_x000a_" dataDxfId="20">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r5a9ad54dbed04bbd846d96c703c59258"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="79" xr3:uid="{CA6CF9A1-F0B6-4DEB-9538-F27E190F4122}" name="Nome do servidor11" dataDxfId="19">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="rbb8c6a6e892f49e48cc88813b848b152"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="80" xr3:uid="{67879B6C-8E31-491D-9AC6-0A2CBD6A6C16}" name="Matrícula do servidor11" dataDxfId="18">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="re5b8a05b8de54e5cac4532075bab19ed"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="81" xr3:uid="{9403AE86-B7C7-40E6-8060-2403D63E37AF}" name="Login de rede11" dataDxfId="17">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r8a8f0e3373944cb78bccc73ba7287f3e"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="82" xr3:uid="{FE872543-AFAF-4394-83AD-1AA92CFA8F41}" name="E-mail institucional11" dataDxfId="16">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r41a461a380cf4014b5de40d947afd792"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="83" xr3:uid="{00A04EDD-754D-4796-8235-2EAE5A29602F}" name="Coordenação do servidor10" dataDxfId="15">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r0a43abf457ad454ca17fcb5223903741"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="84" xr3:uid="{0AB3FD6A-B0DA-4826-837F-D2EE1A5CDEB5}" name="Nome do servidor12" dataDxfId="14">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r07c18bbdfb154e39b975dc9c46d2007b"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="85" xr3:uid="{AE8F53D5-3142-4B9D-8F32-C7B9C505FB7B}" name="Matrícula do servidor12" dataDxfId="13">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r602268d11a3a4ad1bb31b9df47b3e4b9"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="86" xr3:uid="{5493D1AA-D3D7-48D2-AEA2-ECFA5CAE976A}" name="Login de rede12" dataDxfId="12">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r7cc89ab1087d45b0b370c49f4d553ee7"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="87" xr3:uid="{C5C09E6A-A926-41CF-96BF-981B8D4C5D92}" name="E-mail institucional14" dataDxfId="11">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r2b0af254dd35464aaacc2d2d78e24b8c"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="88" xr3:uid="{85290EF9-84DF-414B-92B8-165B47BE44D5}" name="Coordenação do servidor12" dataDxfId="10">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="raeab11e9c9944e0e97921cca9115a830"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="89" xr3:uid="{924EC870-B502-4586-9558-5A43D47B52B6}" name="Nome do servidor13" dataDxfId="9">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r9fe65917f55a4510a00da38005fe4cfb"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="90" xr3:uid="{7DE4E560-FB53-46A7-9470-623AC0B0EA55}" name="Matrícula do servidor13" dataDxfId="8">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r9c125fed12964f35a28b2f00d386bad3"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="91" xr3:uid="{5BE2C3F2-4C9B-41C6-9475-9DC280A90506}" name="Login de rede13" dataDxfId="7">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r8e4202475e5f4af48dd1614e1cefd060"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="92" xr3:uid="{19188253-6386-4678-B917-50200E0C83E1}" name="E-mail institucional12" dataDxfId="6">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="rdf0677a62aec4c798d8909db39276164"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="93" xr3:uid="{8FE6AE0F-7FCD-4CA4-BFB6-11BD6470134E}" name="Coordenação do servidor_x000a_1" dataDxfId="5">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r8e92128aab04420dba4eb35d0d5b947e"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="94" xr3:uid="{152B27B0-9AA7-4C5A-8548-92E25E08C653}" name="Nome do servidor14" dataDxfId="4">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="r39877476145448d5b94b5d566a37d0f9"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="95" xr3:uid="{2753F683-EEE1-4665-BF88-665EEE639924}" name="Matrícula do servidor14" dataDxfId="3">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="rd4172bd5b8b444c0bec4fbc48cf2569c"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="96" xr3:uid="{A06BB60C-E8B6-4966-A029-0140F77E8575}" name="Login de rede14" dataDxfId="2">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="rda675e28c411417e9c48bc15645340a2"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="97" xr3:uid="{04A33593-60B6-4A0B-AE87-4849C0AB4B67}" name="E-mail institucional13" dataDxfId="1">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="ra8a734903d3e40b7982fc028cdf4e4a3"/>
+        </ext>
+      </extLst>
+    </tableColumn>
+    <tableColumn id="98" xr3:uid="{0BC0A1A3-FBB3-4040-9F5A-D89747687D64}" name="Coordenação do servidor11" dataDxfId="0">
+      <extLst>
+        <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{FCC71383-01E1-4257-9335-427F07BE8D7F}">
+          <xlmsforms:question id="rfab5ed83323e4e5e96fba34632b721f8"/>
         </ext>
       </extLst>
     </tableColumn>
@@ -1426,7 +1792,7 @@
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
     <ext xmlns:xlmsforms="http://schemas.microsoft.com/office/spreadsheetml/2023/msForms" uri="{839C7E11-91E4-4DBD-9C5D-0DEA604FA9AC}">
-      <xlmsforms:msForm id="u0batxyrhEm5RpBzJtLcbwbpCD8piBVKn3szfQGwYEVUM0w1OFNRNkNDV1BORjBYRERXRjBOWUY3Ny4u" isFormConnected="1" maxResponseId="11" latestEventMarker="202">
+      <xlmsforms:msForm id="u0batxyrhEm5RpBzJtLcbwbpCD8piBVKn3szfQGwYEVUM0w1OFNRNkNDV1BORjBYRERXRjBOWUY3Ny4u" isFormConnected="1" maxResponseId="12" latestEventMarker="269">
         <xlmsforms:syncedQuestionId>id</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>startDate</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>submitDate</xlmsforms:syncedQuestionId>
@@ -1500,6 +1866,31 @@
         <xlmsforms:syncedQuestionId>r993ffb00f9924bcbb8f493f7869380b6</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>r2498731ab00f4da28f82ffdb063b6d21</xlmsforms:syncedQuestionId>
         <xlmsforms:syncedQuestionId>r1a9c813d9b0a445d9ce4a40e335039c3</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>rac27fd054e3345469c7b9996b6af173a</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r4256c493215a4a2097426ca815f3afda</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r1a9fbbe7b2244704bb8ecc69f4bffeb4</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r3bcc0c0e808a46169ae8a8ea01caf5d4</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r5a9ad54dbed04bbd846d96c703c59258</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>rbb8c6a6e892f49e48cc88813b848b152</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>re5b8a05b8de54e5cac4532075bab19ed</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r8a8f0e3373944cb78bccc73ba7287f3e</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r41a461a380cf4014b5de40d947afd792</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r0a43abf457ad454ca17fcb5223903741</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r07c18bbdfb154e39b975dc9c46d2007b</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r602268d11a3a4ad1bb31b9df47b3e4b9</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r7cc89ab1087d45b0b370c49f4d553ee7</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r2b0af254dd35464aaacc2d2d78e24b8c</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>raeab11e9c9944e0e97921cca9115a830</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r9fe65917f55a4510a00da38005fe4cfb</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r9c125fed12964f35a28b2f00d386bad3</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r8e4202475e5f4af48dd1614e1cefd060</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>rdf0677a62aec4c798d8909db39276164</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r8e92128aab04420dba4eb35d0d5b947e</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>r39877476145448d5b94b5d566a37d0f9</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>rd4172bd5b8b444c0bec4fbc48cf2569c</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>rda675e28c411417e9c48bc15645340a2</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>ra8a734903d3e40b7982fc028cdf4e4a3</xlmsforms:syncedQuestionId>
+        <xlmsforms:syncedQuestionId>rfab5ed83323e4e5e96fba34632b721f8</xlmsforms:syncedQuestionId>
       </xlmsforms:msForm>
     </ext>
   </extLst>
@@ -1803,16 +2194,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BU12"/>
+  <dimension ref="A1:CT13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="10" width="20" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="19" customWidth="1"/>
     <col min="13" max="16" width="20" bestFit="1" customWidth="1"/>
     <col min="17" max="71" width="19" customWidth="1"/>
+    <col min="74" max="98" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73">
+    <row r="1" spans="1:98" ht="45.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1843,10 +2235,10 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
       <c r="M1" t="s">
@@ -2032,8 +2424,83 @@
       <c r="BU1" t="s">
         <v>72</v>
       </c>
+      <c r="BV1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>74</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>75</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>76</v>
+      </c>
+      <c r="BZ1" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="CA1" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="CB1" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="CC1" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="CD1" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="CE1" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="CF1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="CG1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="CH1" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="CI1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="CJ1" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="CK1" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="CL1" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="CM1" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="CN1" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="CO1" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="CP1" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="CQ1" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="CR1" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="CS1" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="CT1" s="5" t="s">
+        <v>97</v>
+      </c>
     </row>
-    <row r="2" spans="1:73">
+    <row r="2" spans="1:98">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2044,45 +2511,43 @@
         <v>46097.59547453704</v>
       </c>
       <c r="D2" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="F2" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H2" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="I2" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="J2" t="s">
-        <v>78</v>
-      </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
+        <v>103</v>
+      </c>
       <c r="M2" s="1" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="N2" t="s">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="P2" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="Q2" t="s">
-        <v>83</v>
+        <v>108</v>
       </c>
       <c r="R2" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:73">
+    <row r="3" spans="1:98">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2093,45 +2558,43 @@
         <v>46097.596122685187</v>
       </c>
       <c r="D3" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H3" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="I3" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="J3" t="s">
-        <v>84</v>
-      </c>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
+        <v>109</v>
+      </c>
       <c r="M3" s="1" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="N3" t="s">
-        <v>85</v>
+        <v>110</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="P3" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
       <c r="Q3" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="R3" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:73">
+    <row r="4" spans="1:98">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2142,45 +2605,43 @@
         <v>46097.596689814818</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H4" t="s">
-        <v>76</v>
+        <v>101</v>
       </c>
       <c r="I4" t="s">
-        <v>77</v>
+        <v>102</v>
       </c>
       <c r="J4" t="s">
-        <v>84</v>
-      </c>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
+        <v>109</v>
+      </c>
       <c r="M4" s="1" t="s">
-        <v>79</v>
+        <v>104</v>
       </c>
       <c r="N4" t="s">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="P4" t="s">
-        <v>91</v>
+        <v>116</v>
       </c>
       <c r="Q4" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="R4" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
     </row>
-    <row r="5" spans="1:73">
+    <row r="5" spans="1:98">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2191,46 +2652,44 @@
         <v>46097.682604166701</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="J5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="N5" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>74</v>
-      </c>
       <c r="O5" s="4" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:73">
+    <row r="6" spans="1:98">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2241,46 +2700,44 @@
         <v>46097.683113425897</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="M6" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="K6" s="5"/>
-      <c r="L6" s="5"/>
-      <c r="M6" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="N6" s="3" t="s">
-        <v>108</v>
+        <v>133</v>
       </c>
       <c r="O6" s="4" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="R6" s="3" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:73">
+    <row r="7" spans="1:98">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2291,46 +2748,44 @@
         <v>46097.692893518499</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
+        <v>124</v>
+      </c>
       <c r="M7" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="O7" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="O7" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="P7" s="3" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
       <c r="R7" s="3" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
     </row>
-    <row r="8" spans="1:73">
+    <row r="8" spans="1:98">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2341,121 +2796,119 @@
         <v>46099.424282407403</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3" t="s">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>117</v>
+        <v>142</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>118</v>
+        <v>143</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="K8" s="5"/>
-      <c r="L8" s="5"/>
+        <v>144</v>
+      </c>
       <c r="M8" s="4" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="O8" s="4" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="R8" s="3" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="S8" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="T8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="U8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="V8" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="W8" t="s">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="X8" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="Y8" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="Z8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AA8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AB8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AC8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AD8" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="AE8" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="AF8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AG8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AH8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AI8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AJ8" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="AK8" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="AL8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AM8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AN8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AO8" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="AP8" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="AQ8" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
     </row>
-    <row r="9" spans="1:73">
+    <row r="9" spans="1:98">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2466,67 +2919,65 @@
         <v>46099.426805555602</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3" t="s">
-        <v>127</v>
+        <v>152</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="K9" s="5"/>
-      <c r="L9" s="5"/>
+        <v>153</v>
+      </c>
       <c r="M9" s="4" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="N9" s="3" t="s">
-        <v>121</v>
+        <v>146</v>
       </c>
       <c r="O9" s="4" t="s">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="R9" s="3" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="S9" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="T9" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="U9" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="V9" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
       <c r="W9" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="X9" t="s">
-        <v>136</v>
+        <v>161</v>
       </c>
       <c r="Y9" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:73">
+    <row r="10" spans="1:98">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2537,85 +2988,83 @@
         <v>46099.428553240701</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3" t="s">
-        <v>137</v>
+        <v>162</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>138</v>
+        <v>163</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>139</v>
+        <v>164</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
+        <v>99</v>
+      </c>
       <c r="M10" s="4" t="s">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>141</v>
+        <v>166</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>142</v>
+        <v>167</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>133</v>
+        <v>158</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>143</v>
+        <v>168</v>
       </c>
       <c r="S10" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="T10" t="s">
-        <v>144</v>
+        <v>169</v>
       </c>
       <c r="U10" t="s">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="V10" t="s">
-        <v>146</v>
+        <v>171</v>
       </c>
       <c r="W10" t="s">
+        <v>172</v>
+      </c>
+      <c r="X10" t="s">
+        <v>173</v>
+      </c>
+      <c r="Y10" t="s">
         <v>147</v>
       </c>
-      <c r="X10" t="s">
-        <v>148</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>122</v>
-      </c>
       <c r="Z10" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
       <c r="AA10" t="s">
-        <v>150</v>
+        <v>175</v>
       </c>
       <c r="AB10" t="s">
+        <v>176</v>
+      </c>
+      <c r="AC10" t="s">
+        <v>177</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>178</v>
+      </c>
+      <c r="AE10" t="s">
         <v>151</v>
       </c>
-      <c r="AC10" t="s">
-        <v>152</v>
-      </c>
-      <c r="AD10" t="s">
-        <v>153</v>
-      </c>
-      <c r="AE10" t="s">
-        <v>126</v>
-      </c>
     </row>
-    <row r="11" spans="1:73">
+    <row r="11" spans="1:98">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2626,158 +3075,156 @@
         <v>46099.439490740697</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3" t="s">
-        <v>154</v>
+        <v>179</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>116</v>
+        <v>141</v>
       </c>
       <c r="H11" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="M11" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="R11" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="S11" t="s">
+        <v>147</v>
+      </c>
+      <c r="T11" t="s">
+        <v>188</v>
+      </c>
+      <c r="U11" t="s">
+        <v>189</v>
+      </c>
+      <c r="V11" t="s">
+        <v>190</v>
+      </c>
+      <c r="W11" t="s">
+        <v>191</v>
+      </c>
+      <c r="X11" t="s">
+        <v>139</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>147</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>192</v>
+      </c>
+      <c r="AA11" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="AB11" t="s">
         <v>155</v>
       </c>
-      <c r="I11" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="O11" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="P11" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q11" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="R11" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="S11" t="s">
-        <v>122</v>
-      </c>
-      <c r="T11" t="s">
-        <v>163</v>
-      </c>
-      <c r="U11" t="s">
-        <v>164</v>
-      </c>
-      <c r="V11" t="s">
-        <v>165</v>
-      </c>
-      <c r="W11" t="s">
-        <v>166</v>
-      </c>
-      <c r="X11" t="s">
-        <v>114</v>
-      </c>
-      <c r="Y11" t="s">
-        <v>122</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>167</v>
-      </c>
-      <c r="AA11" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>130</v>
-      </c>
       <c r="AC11" t="s">
-        <v>168</v>
+        <v>193</v>
       </c>
       <c r="AD11" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="AE11" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="AF11" t="s">
-        <v>169</v>
+        <v>194</v>
       </c>
       <c r="AG11" s="1" t="s">
-        <v>170</v>
+        <v>195</v>
       </c>
       <c r="AH11" s="1" t="s">
-        <v>171</v>
+        <v>196</v>
       </c>
       <c r="AI11" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
       <c r="AJ11" t="s">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="AK11" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="AL11" t="s">
-        <v>173</v>
+        <v>198</v>
       </c>
       <c r="AM11" s="1" t="s">
-        <v>174</v>
+        <v>199</v>
       </c>
       <c r="AN11" t="s">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="AO11" t="s">
-        <v>176</v>
+        <v>201</v>
       </c>
       <c r="AP11" t="s">
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="AQ11" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="AR11" t="s">
-        <v>177</v>
+        <v>202</v>
       </c>
       <c r="AS11" s="1" t="s">
-        <v>178</v>
+        <v>203</v>
       </c>
       <c r="AT11" t="s">
-        <v>179</v>
+        <v>204</v>
       </c>
       <c r="AU11" t="s">
-        <v>180</v>
+        <v>205</v>
       </c>
       <c r="AV11" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="AW11" t="s">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="AX11" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
       <c r="AY11" s="1" t="s">
-        <v>182</v>
+        <v>207</v>
       </c>
       <c r="AZ11" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
       <c r="BA11" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
       <c r="BB11" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="BC11" t="s">
-        <v>126</v>
+        <v>151</v>
       </c>
     </row>
-    <row r="12" spans="1:73">
-      <c r="A12" s="5">
+    <row r="12" spans="1:98">
+      <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" s="2">
@@ -2787,117 +3234,223 @@
         <v>46101.612800925897</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>94</v>
+        <v>119</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3" t="s">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>185</v>
+        <v>210</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>186</v>
+        <v>211</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>187</v>
+        <v>212</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="K12" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="L12" s="5" t="s">
-        <v>189</v>
+        <v>213</v>
+      </c>
+      <c r="K12" t="s">
+        <v>147</v>
+      </c>
+      <c r="L12" t="s">
+        <v>214</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="N12" s="3" t="s">
-        <v>191</v>
+        <v>216</v>
       </c>
       <c r="O12" s="4" t="s">
-        <v>192</v>
+        <v>217</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>132</v>
+        <v>157</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>131</v>
+        <v>156</v>
       </c>
       <c r="R12" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="S12" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="T12" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="U12" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="V12" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="W12" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="X12" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="Y12" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="Z12" s="5"/>
-      <c r="AA12" s="6"/>
-      <c r="AB12" s="5"/>
-      <c r="AC12" s="5"/>
-      <c r="AD12" s="5"/>
-      <c r="AE12" s="5"/>
-      <c r="AF12" s="5"/>
-      <c r="AG12" s="6"/>
-      <c r="AH12" s="6"/>
-      <c r="AI12" s="5"/>
-      <c r="AJ12" s="5"/>
-      <c r="AK12" s="5"/>
-      <c r="AL12" s="5"/>
-      <c r="AM12" s="6"/>
-      <c r="AN12" s="5"/>
-      <c r="AO12" s="5"/>
-      <c r="AP12" s="5"/>
-      <c r="AQ12" s="5"/>
-      <c r="AR12" s="5"/>
-      <c r="AS12" s="6"/>
-      <c r="AT12" s="5"/>
-      <c r="AU12" s="5"/>
-      <c r="AV12" s="5"/>
-      <c r="AW12" s="5"/>
-      <c r="AX12" s="5"/>
-      <c r="AY12" s="6"/>
-      <c r="AZ12" s="5"/>
-      <c r="BA12" s="5"/>
-      <c r="BB12" s="5"/>
-      <c r="BC12" s="5"/>
-      <c r="BD12" s="5"/>
-      <c r="BE12" s="5"/>
-      <c r="BF12" s="5"/>
-      <c r="BG12" s="5"/>
-      <c r="BH12" s="5"/>
-      <c r="BI12" s="5"/>
-      <c r="BJ12" s="5"/>
-      <c r="BK12" s="5"/>
-      <c r="BL12" s="5"/>
-      <c r="BM12" s="5"/>
-      <c r="BN12" s="5"/>
-      <c r="BO12" s="5"/>
-      <c r="BP12" s="5"/>
-      <c r="BQ12" s="5"/>
-      <c r="BR12" s="5"/>
-      <c r="BS12" s="5"/>
-      <c r="BT12" s="5"/>
-      <c r="BU12" s="5"/>
+        <v>218</v>
+      </c>
+      <c r="S12" t="s">
+        <v>147</v>
+      </c>
+      <c r="T12" t="s">
+        <v>219</v>
+      </c>
+      <c r="U12" t="s">
+        <v>220</v>
+      </c>
+      <c r="V12" t="s">
+        <v>221</v>
+      </c>
+      <c r="W12" t="s">
+        <v>222</v>
+      </c>
+      <c r="X12" t="s">
+        <v>223</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>151</v>
+      </c>
+      <c r="AA12" s="1"/>
+      <c r="AG12" s="1"/>
+      <c r="AH12" s="1"/>
+      <c r="AM12" s="1"/>
+      <c r="AS12" s="1"/>
+      <c r="AY12" s="1"/>
+    </row>
+    <row r="13" spans="1:98">
+      <c r="A13" s="6">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2">
+        <v>46104.486331018503</v>
+      </c>
+      <c r="C13" s="2">
+        <v>46104.488414351901</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="P13" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="Q13" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="R13" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="S13" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="T13" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="U13" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="V13" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="W13" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="X13" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="Y13" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="Z13" s="6"/>
+      <c r="AA13" s="7"/>
+      <c r="AB13" s="6"/>
+      <c r="AC13" s="6"/>
+      <c r="AD13" s="6"/>
+      <c r="AE13" s="6"/>
+      <c r="AF13" s="6"/>
+      <c r="AG13" s="7"/>
+      <c r="AH13" s="7"/>
+      <c r="AI13" s="6"/>
+      <c r="AJ13" s="6"/>
+      <c r="AK13" s="6"/>
+      <c r="AL13" s="6"/>
+      <c r="AM13" s="7"/>
+      <c r="AN13" s="6"/>
+      <c r="AO13" s="6"/>
+      <c r="AP13" s="6"/>
+      <c r="AQ13" s="6"/>
+      <c r="AR13" s="6"/>
+      <c r="AS13" s="7"/>
+      <c r="AT13" s="6"/>
+      <c r="AU13" s="6"/>
+      <c r="AV13" s="6"/>
+      <c r="AW13" s="6"/>
+      <c r="AX13" s="6"/>
+      <c r="AY13" s="7"/>
+      <c r="AZ13" s="6"/>
+      <c r="BA13" s="6"/>
+      <c r="BB13" s="6"/>
+      <c r="BC13" s="6"/>
+      <c r="BD13" s="6"/>
+      <c r="BE13" s="6"/>
+      <c r="BF13" s="6"/>
+      <c r="BG13" s="6"/>
+      <c r="BH13" s="6"/>
+      <c r="BI13" s="6"/>
+      <c r="BJ13" s="6"/>
+      <c r="BK13" s="6"/>
+      <c r="BL13" s="6"/>
+      <c r="BM13" s="6"/>
+      <c r="BN13" s="6"/>
+      <c r="BO13" s="6"/>
+      <c r="BP13" s="6"/>
+      <c r="BQ13" s="6"/>
+      <c r="BR13" s="6"/>
+      <c r="BS13" s="6"/>
+      <c r="BT13" s="6"/>
+      <c r="BU13" s="6"/>
+      <c r="BV13" s="6"/>
+      <c r="BW13" s="6"/>
+      <c r="BX13" s="6"/>
+      <c r="BY13" s="6"/>
+      <c r="BZ13" s="6"/>
+      <c r="CA13" s="6"/>
+      <c r="CB13" s="6"/>
+      <c r="CC13" s="6"/>
+      <c r="CD13" s="6"/>
+      <c r="CE13" s="6"/>
+      <c r="CF13" s="6"/>
+      <c r="CG13" s="6"/>
+      <c r="CH13" s="6"/>
+      <c r="CI13" s="6"/>
+      <c r="CJ13" s="6"/>
+      <c r="CK13" s="6"/>
+      <c r="CL13" s="6"/>
+      <c r="CM13" s="6"/>
+      <c r="CN13" s="6"/>
+      <c r="CO13" s="6"/>
+      <c r="CP13" s="6"/>
+      <c r="CQ13" s="6"/>
+      <c r="CR13" s="6"/>
+      <c r="CS13" s="6"/>
+      <c r="CT13" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>